<commit_message>
feat(ultrafast): cap nhat text loi SDT + sync rule + ket qua run
- BA doi text loi SDT sai dinh dang: "So dien thoai khong hop le."
  -> "So dien thoai chua dung, moi nhap lai" (SC-006, SC-007)
- Cap nhat TC Excel (TC_DANGKYUF.7/.8) + dong bo assertion automation
  (spec.ts + page.ts) theo requirement, khong de code tu khop UI
- sync-tc-results: codify rule skip = Block + ly do, note ngay thuc hien
  vao cot Ghi Chu (L), map cot I/J/K/L chinh xac
- Ket qua run 2026-05-30: 17 Pass / 3 Fail / 8 Block
  + DEFECT-DANGKYUF-001: staging hien COD trai SC-011 (BA xac nhan no COD)

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ecom-pdh/03_test-cases/AI_ISC_ecom-pdh_v1.1_TC_v1.0.xlsx
+++ b/ecom-pdh/03_test-cases/AI_ISC_ecom-pdh_v1.1_TC_v1.0.xlsx
@@ -86,7 +86,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -116,6 +116,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00A9D08E"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFF2CC"/>
       </patternFill>
     </fill>
   </fills>
@@ -386,7 +391,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -465,6 +470,21 @@
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="7" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="7" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="7" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2537,106 +2557,114 @@
       <c r="L16" s="36" t="inlineStr"/>
     </row>
     <row r="17" ht="80" customHeight="1" s="2">
-      <c r="A17" s="33" t="inlineStr">
-        <is>
-          <t>AI</t>
-        </is>
-      </c>
-      <c r="B17" s="34" t="inlineStr">
+      <c r="A17" s="37" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="B17" s="38" t="inlineStr">
         <is>
           <t>TC_DANGKYUF.7</t>
         </is>
       </c>
-      <c r="C17" s="34" t="inlineStr">
+      <c r="C17" s="38" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="D17" s="35" t="inlineStr">
+      <c r="D17" s="39" t="inlineStr">
         <is>
           <t>Kiểm tra báo lỗi khi nhập Số điện thoại ít hơn 10 số</t>
         </is>
       </c>
-      <c r="E17" s="35" t="inlineStr">
+      <c r="E17" s="39" t="inlineStr">
         <is>
           <t>- Đang ở màn hình Checkout UltraFast
 - Trường Số điện thoại đang trống
 Dữ liệu test: SĐT 9 số (VD: 090123456)</t>
         </is>
       </c>
-      <c r="F17" s="35" t="inlineStr">
+      <c r="F17" s="39" t="inlineStr">
         <is>
           <t>1. Click vào trường "Số điện thoại"
 2. Nhập SĐT 9 số (VD: 090123456)
 3. Click ra ngoài trường hoặc click button "Thanh toán"</t>
         </is>
       </c>
-      <c r="G17" s="35" t="inlineStr">
-        <is>
-          <t>- Hiển thị thông báo lỗi: "Số điện thoại không hợp lệ."
+      <c r="G17" s="39" t="inlineStr">
+        <is>
+          <t>- Hiển thị thông báo lỗi: "Số điện thoại chưa đúng, mời nhập lại"
 - Border đỏ xuất hiện quanh textbox</t>
         </is>
       </c>
-      <c r="H17" s="36" t="inlineStr">
+      <c r="H17" s="40" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
       <c r="I17" s="36" t="inlineStr"/>
       <c r="J17" s="36" t="inlineStr"/>
-      <c r="K17" s="36" t="inlineStr"/>
-      <c r="L17" s="36" t="inlineStr"/>
+      <c r="K17" s="41" t="n"/>
+      <c r="L17" s="41" t="inlineStr">
+        <is>
+          <t>Update: BA đổi text lỗi SĐT sai định dạng "Số điện thoại không hợp lệ." -&gt; "Số điện thoại chưa đúng, mời nhập lại" (2026-05-30)</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="80" customHeight="1" s="2">
-      <c r="A18" s="33" t="inlineStr">
-        <is>
-          <t>AI</t>
-        </is>
-      </c>
-      <c r="B18" s="34" t="inlineStr">
+      <c r="A18" s="37" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="B18" s="38" t="inlineStr">
         <is>
           <t>TC_DANGKYUF.8</t>
         </is>
       </c>
-      <c r="C18" s="34" t="inlineStr">
+      <c r="C18" s="38" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="D18" s="35" t="inlineStr">
+      <c r="D18" s="39" t="inlineStr">
         <is>
           <t>Kiểm tra báo lỗi khi nhập Số điện thoại không bắt đầu bằng 0</t>
         </is>
       </c>
-      <c r="E18" s="35" t="inlineStr">
+      <c r="E18" s="39" t="inlineStr">
         <is>
           <t>- Đang ở màn hình Checkout UltraFast
 - Trường Số điện thoại đang trống
 Dữ liệu test: SĐT 10 số bắt đầu bằng 1 (VD: 1901234567)</t>
         </is>
       </c>
-      <c r="F18" s="35" t="inlineStr">
+      <c r="F18" s="39" t="inlineStr">
         <is>
           <t>1. Click vào trường "Số điện thoại"
 2. Nhập SĐT 10 số không bắt đầu bằng 0 (VD: 1901234567)
 3. Click ra ngoài trường hoặc click "Thanh toán"</t>
         </is>
       </c>
-      <c r="G18" s="35" t="inlineStr">
-        <is>
-          <t>- Hiển thị thông báo lỗi: "Số điện thoại không hợp lệ."
+      <c r="G18" s="39" t="inlineStr">
+        <is>
+          <t>- Hiển thị thông báo lỗi: "Số điện thoại chưa đúng, mời nhập lại"
 - Border đỏ xuất hiện quanh textbox</t>
         </is>
       </c>
-      <c r="H18" s="36" t="inlineStr">
+      <c r="H18" s="40" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
       <c r="I18" s="36" t="inlineStr"/>
       <c r="J18" s="36" t="inlineStr"/>
-      <c r="K18" s="36" t="inlineStr"/>
-      <c r="L18" s="36" t="inlineStr"/>
+      <c r="K18" s="41" t="n"/>
+      <c r="L18" s="41" t="inlineStr">
+        <is>
+          <t>Update: BA đổi text lỗi SĐT sai định dạng "Số điện thoại không hợp lệ." -&gt; "Số điện thoại chưa đúng, mời nhập lại" (2026-05-30)</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="80" customHeight="1" s="2">
       <c r="A19" s="33" t="inlineStr">

</xml_diff>